<commit_message>
Fix reimbursement export state and templates
</commit_message>
<xml_diff>
--- a/web/public/templates/korea_reimbursement_template.xlsx
+++ b/web/public/templates/korea_reimbursement_template.xlsx
@@ -734,22 +734,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <authors>
-    <author>admin</author>
-  </authors>
-  <commentList>
-    <comment ref="J2" authorId="0" shapeId="0">
-      <text>
-        <t>记得找仓库管理员“汪东跃”入库哦
-然后再来找财务报销</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2123,7 +2107,6 @@
     <mergeCell ref="A35:B35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Remove frozen pane from Korea details
</commit_message>
<xml_diff>
--- a/web/public/templates/korea_reimbursement_template.xlsx
+++ b/web/public/templates/korea_reimbursement_template.xlsx
@@ -1188,15 +1188,15 @@
   <mergeCells count="14">
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="G3:I4"/>
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A11:I11"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="F10:G10"/>
     <mergeCell ref="H10:I10"/>
-    <mergeCell ref="A9:B9"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="G3:I4"/>
+    <mergeCell ref="A9:B9"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="A3:B3"/>
     <mergeCell ref="A6:B6"/>
@@ -1215,24 +1215,24 @@
   <dimension ref="A1:T35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14.69921875" customWidth="1" min="1" max="1"/>
-    <col width="39.796875" customWidth="1" min="2" max="2"/>
-    <col width="31.09765625" customWidth="1" min="3" max="3"/>
-    <col width="15.3984375" customWidth="1" min="4" max="4"/>
-    <col width="19.296875" customWidth="1" min="5" max="5"/>
-    <col width="35.796875" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="10.796875" customWidth="1" min="8" max="8"/>
-    <col width="26.59765625" customWidth="1" min="10" max="10"/>
-    <col width="21" customWidth="1" min="11" max="11"/>
-    <col width="10.3984375" bestFit="1" customWidth="1" min="12" max="12"/>
-    <col width="21.296875" customWidth="1" min="13" max="13"/>
-    <col width="9.59765625" customWidth="1" min="14" max="14"/>
-    <col width="21" customWidth="1" min="15" max="15"/>
-    <col width="10.3984375" bestFit="1" customWidth="1" min="16" max="16"/>
-    <col width="18.296875" customWidth="1" min="17" max="17"/>
-    <col width="15.5" customWidth="1" min="18" max="18"/>
-    <col width="17" customWidth="1" min="19" max="19"/>
+    <col width="14.69921875" customWidth="1" style="27" min="1" max="1"/>
+    <col width="39.796875" customWidth="1" style="27" min="2" max="2"/>
+    <col width="31.09765625" customWidth="1" style="27" min="3" max="3"/>
+    <col width="15.3984375" customWidth="1" style="27" min="4" max="4"/>
+    <col width="19.296875" customWidth="1" style="27" min="5" max="5"/>
+    <col width="35.796875" customWidth="1" style="27" min="6" max="6"/>
+    <col width="8" customWidth="1" style="27" min="7" max="7"/>
+    <col width="10.796875" customWidth="1" style="27" min="8" max="8"/>
+    <col width="26.59765625" customWidth="1" style="27" min="10" max="10"/>
+    <col width="21" customWidth="1" style="27" min="11" max="11"/>
+    <col width="10.3984375" bestFit="1" customWidth="1" style="27" min="12" max="12"/>
+    <col width="21.296875" customWidth="1" style="27" min="13" max="13"/>
+    <col width="9.59765625" customWidth="1" style="27" min="14" max="14"/>
+    <col width="21" customWidth="1" style="27" min="15" max="15"/>
+    <col width="10.3984375" bestFit="1" customWidth="1" style="27" min="16" max="16"/>
+    <col width="18.296875" customWidth="1" style="27" min="17" max="17"/>
+    <col width="15.5" customWidth="1" style="27" min="18" max="18"/>
+    <col width="17" customWidth="1" style="27" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1245,7 +1245,7 @@
       <c r="S1" s="41" t="n"/>
       <c r="T1" s="42" t="n"/>
     </row>
-    <row r="2" ht="124.45" customHeight="1">
+    <row r="2" ht="124.45" customHeight="1" s="27">
       <c r="A2" s="43" t="inlineStr">
         <is>
           <t>日期
@@ -1358,7 +1358,7 @@
       </c>
       <c r="T2" s="42" t="n"/>
     </row>
-    <row r="3" ht="31.1" customHeight="1">
+    <row r="3" ht="31.1" customHeight="1" s="27">
       <c r="A3" s="48" t="n"/>
       <c r="B3" s="49" t="n"/>
       <c r="C3" s="49" t="n"/>
@@ -2040,7 +2040,7 @@
       <c r="S33" s="56" t="n"/>
       <c r="T33" s="42" t="n"/>
     </row>
-    <row r="34" ht="35.45" customHeight="1">
+    <row r="34" ht="35.45" customHeight="1" s="27">
       <c r="A34" s="84" t="inlineStr">
         <is>
           <t>合计（外币）
@@ -2070,7 +2070,7 @@
       <c r="S34" s="56" t="n"/>
       <c r="T34" s="42" t="n"/>
     </row>
-    <row r="35" ht="50.4" customHeight="1">
+    <row r="35" ht="50.4" customHeight="1" s="27">
       <c r="A35" s="89" t="inlineStr">
         <is>
           <t>合计（人民币）

</xml_diff>